<commit_message>
Add Solgar brand (10 products + banner), NOW Kids Echinacea, ECOVITA Chlorophyll; link price list
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/YOSHLIK-YU - Price ORIGINAL....xlsx
+++ b/YOSHLIK-YU - Price ORIGINAL....xlsx
@@ -4077,7 +4077,7 @@
           <t>N F</t>
         </is>
       </c>
-      <c r="C60" s="129" t="inlineStr">
+      <c r="C60" s="144" t="inlineStr">
         <is>
           <t>C-1000 с шиповником, 100 таблеток</t>
         </is>
@@ -5663,7 +5663,7 @@
           <t>N F</t>
         </is>
       </c>
-      <c r="C94" s="61" t="inlineStr">
+      <c r="C94" s="143" t="inlineStr">
         <is>
           <t>Детский Жидкая эхинацея, апельсин,  59 мл</t>
         </is>
@@ -10623,7 +10623,7 @@
           <t>E V</t>
         </is>
       </c>
-      <c r="C207" s="129" t="inlineStr">
+      <c r="C207" s="144" t="inlineStr">
         <is>
           <t>Жидкий хлорофилл c ароматом натуральной мяты, 500 мл</t>
         </is>
@@ -11175,9 +11175,6 @@
       <c r="M221" s="2" t="n"/>
       <c r="N221" s="1" t="n"/>
     </row>
-    <row r="222"/>
-    <row r="223"/>
-    <row r="224"/>
     <row r="225" customFormat="1" s="10">
       <c r="A225" s="1" t="n"/>
       <c r="B225" s="19" t="n"/>
@@ -11210,8 +11207,6 @@
       <c r="M226" s="2" t="n"/>
       <c r="N226" s="1" t="n"/>
     </row>
-    <row r="227"/>
-    <row r="228"/>
     <row r="229" customFormat="1" s="8">
       <c r="A229" s="1" t="n"/>
       <c r="B229" s="19" t="n"/>
@@ -11244,8 +11239,6 @@
       <c r="M230" s="2" t="n"/>
       <c r="N230" s="1" t="n"/>
     </row>
-    <row r="231"/>
-    <row r="232"/>
     <row r="233" customFormat="1" s="8">
       <c r="A233" s="1" t="n"/>
       <c r="B233" s="19" t="n"/>
@@ -11262,9 +11255,6 @@
       <c r="M233" s="2" t="n"/>
       <c r="N233" s="1" t="n"/>
     </row>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
     <row r="237" customFormat="1" s="10">
       <c r="A237" s="1" t="n"/>
       <c r="B237" s="19" t="n"/>
@@ -11342,154 +11332,157 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C58" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C61" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C62" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C65" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C66" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C67" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C68" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C69" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C70" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C71" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C72" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C73" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C74" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C75" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C76" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C77" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C78" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C79" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C80" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C81" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C82" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C83" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C84" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C85" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C86" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C88" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C89" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C90" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C91" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C92" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C93" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C95" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C96" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C97" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C98" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C99" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C100" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C102" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C103" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C104" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C105" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C106" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C107" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C108" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C109" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C111" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C112" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C113" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C114" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C115" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C116" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C117" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C118" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C119" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C120" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C121" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C122" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C123" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C124" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C125" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C126" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C128" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C129" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C130" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C131" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C132" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C133" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C134" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C136" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C137" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C138" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C139" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C140" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C141" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C142" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C144" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C145" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C146" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C147" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C149" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C150" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C151" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C152" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C153" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C154" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C155" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C156" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C157" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C158" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C159" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C160" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C161" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C162" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C163" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C165" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C166" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C167" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C168" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C169" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C170" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C171" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C172" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C173" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C174" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C175" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C176" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C177" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C179" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C180" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C181" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C182" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C183" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C184" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C185" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C186" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C187" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C188" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C189" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C190" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C191" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C192" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C193" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C194" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C195" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C196" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C197" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C198" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C199" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C200" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C201" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C202" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C203" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C204" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C205" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C206" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C211" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C212" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C213" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C214" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C215" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C216" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C217" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C218" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C60" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C61" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C62" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C65" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C66" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C67" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C68" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C69" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C70" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C71" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C72" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C73" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C74" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C75" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C76" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C77" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C78" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C79" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C80" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C81" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C82" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C83" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C84" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C85" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C86" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C88" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C89" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C90" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C91" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C92" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C93" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C94" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C95" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C96" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C97" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C98" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C99" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C100" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C102" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C103" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C104" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C105" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C106" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C107" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C108" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C109" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C111" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C112" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C113" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C114" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C115" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C116" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C117" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C118" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C119" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C120" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C121" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C122" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C123" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C124" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C125" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C126" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C128" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C129" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C130" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C131" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C132" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C133" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C134" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C136" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C137" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C138" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C139" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C140" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C141" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C142" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C144" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C145" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C146" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C147" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C149" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C150" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C151" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C152" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C153" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C154" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C155" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C156" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C157" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C158" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C159" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C160" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C161" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C162" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C163" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C165" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C166" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C167" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C168" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C169" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C170" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C171" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C172" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C173" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C174" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C175" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C176" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C177" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C179" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C180" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C181" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C182" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C183" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C184" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C185" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C186" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C187" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C188" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C189" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C190" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C191" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C192" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C193" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C194" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C195" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C196" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C197" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C198" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C199" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C200" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C201" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C202" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C203" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C204" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C205" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C206" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C207" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C211" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C212" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C213" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C214" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C215" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C216" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C217" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C218" r:id="rId202"/>
   </hyperlinks>
   <pageMargins left="0.39375" right="0.39375" top="0.39375" bottom="0.39375" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" pageOrder="overThenDown" horizontalDpi="300" verticalDpi="300"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId200"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId203"/>
 </worksheet>
 </file>
 

</xml_diff>